<commit_message>
Bill of Materials Updated
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASHUTOSH\Desktop\PCB Projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E0AD17-5449-4CD6-8272-A2E87EF1BCA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB878731-7795-459B-9F29-C1BF1556CE66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{70FA5656-9FE8-4117-A3B6-17E4E3D44C13}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="168">
   <si>
     <t>S.No.</t>
   </si>
@@ -529,6 +529,15 @@
   </si>
   <si>
     <t>USB-C receptacle</t>
+  </si>
+  <si>
+    <t>R_EN</t>
+  </si>
+  <si>
+    <t>EN pull up resistor</t>
+  </si>
+  <si>
+    <t>EN pin to +3V3, required for ESP32 to boot</t>
   </si>
 </sst>
 </file>
@@ -638,7 +647,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -675,6 +684,16 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -990,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56CB1995-C714-481D-8279-82B993E62761}">
-  <dimension ref="A4:G44"/>
+  <dimension ref="A4:G45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" customWidth="1"/>
@@ -1873,6 +1892,26 @@
       </c>
       <c r="G44" s="7" t="s">
         <v>151</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.5">
+      <c r="B45" s="15">
+        <v>41</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="D45" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="E45" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F45" s="17">
+        <v>1</v>
+      </c>
+      <c r="G45" s="18" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>